<commit_message>
add: notes from nations and theirs politics
</commit_message>
<xml_diff>
--- a/Unusual words.xlsx
+++ b/Unusual words.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\InternationalRelations\International relations- notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB73B83B-CF06-4C8E-BB0A-7DB343294D78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{025A7FEE-6A81-46C6-814B-70EA47C52CCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-27240" yWindow="1620" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>juxtaposition</t>
   </si>
@@ -165,6 +165,12 @@
   </si>
   <si>
     <t>odpoczynek</t>
+  </si>
+  <si>
+    <t>conflagration</t>
+  </si>
+  <si>
+    <t>pożoga</t>
   </si>
 </sst>
 </file>
@@ -496,7 +502,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:E8"/>
+  <dimension ref="B1:E9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="21.7109375" customWidth="1"/>
@@ -581,6 +587,14 @@
         <v>19</v>
       </c>
     </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
wip The Nexus reading
</commit_message>
<xml_diff>
--- a/Unusual words.xlsx
+++ b/Unusual words.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\InternationalRelations\International relations- notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{025A7FEE-6A81-46C6-814B-70EA47C52CCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3F279EC-8102-46CB-A1E4-CE691267A9B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27240" yWindow="1620" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>juxtaposition</t>
   </si>
@@ -171,13 +171,34 @@
   </si>
   <si>
     <t>pożoga</t>
+  </si>
+  <si>
+    <t>parsimony</t>
+  </si>
+  <si>
+    <t>skąpstwo</t>
+  </si>
+  <si>
+    <t>unparsimonious</t>
+  </si>
+  <si>
+    <t>nieoszczędny</t>
+  </si>
+  <si>
+    <t>Sprawczość</t>
+  </si>
+  <si>
+    <t>Power</t>
+  </si>
+  <si>
+    <t>Ability to influence others by coercion (hard power) or charm (soft power)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -192,6 +213,21 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -218,10 +254,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
@@ -502,7 +540,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:E9"/>
+  <dimension ref="B1:E12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="21.7109375" customWidth="1"/>
@@ -512,16 +550,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="4" t="s">
         <v>1</v>
       </c>
     </row>
@@ -595,7 +633,35 @@
         <v>21</v>
       </c>
     </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
How chinesee understand soft power
</commit_message>
<xml_diff>
--- a/Unusual words.xlsx
+++ b/Unusual words.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\InternationalRelations\International relations- notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3F279EC-8102-46CB-A1E4-CE691267A9B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C37206D9-929B-4011-8DF5-ED55F8252867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
+    <sheet name="Arkusz2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="64">
   <si>
     <t>juxtaposition</t>
   </si>
@@ -193,12 +194,117 @@
   <si>
     <t>Ability to influence others by coercion (hard power) or charm (soft power)</t>
   </si>
+  <si>
+    <t>pundits</t>
+  </si>
+  <si>
+    <t>eksperci</t>
+  </si>
+  <si>
+    <t>scholars from Hindi pandit and sanskrit pandita</t>
+  </si>
+  <si>
+    <t>chinese</t>
+  </si>
+  <si>
+    <t>pinyin</t>
+  </si>
+  <si>
+    <t>软实力</t>
+  </si>
+  <si>
+    <t>Ruǎn shílì</t>
+  </si>
+  <si>
+    <t>english</t>
+  </si>
+  <si>
+    <t>Soft Power</t>
+  </si>
+  <si>
+    <t>竞争力</t>
+  </si>
+  <si>
+    <t>Jìngzhēng lì</t>
+  </si>
+  <si>
+    <t>hold the line</t>
+  </si>
+  <si>
+    <t>observe calmly</t>
+  </si>
+  <si>
+    <t>冷静观察</t>
+  </si>
+  <si>
+    <t>Lěngjìng guānchá</t>
+  </si>
+  <si>
+    <t>稳住阵脚</t>
+  </si>
+  <si>
+    <t>Wěn zhù zhènjiǎo</t>
+  </si>
+  <si>
+    <t>沉着应对</t>
+  </si>
+  <si>
+    <t>respond calmly</t>
+  </si>
+  <si>
+    <t>Chénzhuó yìngduì</t>
+  </si>
+  <si>
+    <t>善于守拙</t>
+  </si>
+  <si>
+    <t>Shànyú shǒu zhuō</t>
+  </si>
+  <si>
+    <t>Keep a low profile / guard weaknesses</t>
+  </si>
+  <si>
+    <t>决不当- 头</t>
+  </si>
+  <si>
+    <t>Jué bùdāng- tóu</t>
+  </si>
+  <si>
+    <t>Never be a leader</t>
+  </si>
+  <si>
+    <t>attributed to whom</t>
+  </si>
+  <si>
+    <t>Den Xiaoping</t>
+  </si>
+  <si>
+    <t>有所作为</t>
+  </si>
+  <si>
+    <t>Yǒu suǒ zuòwéi</t>
+  </si>
+  <si>
+    <t>Make a difference (from translator) / play your role (from book)</t>
+  </si>
+  <si>
+    <t>韬光养晦</t>
+  </si>
+  <si>
+    <t>Tāoguāngyǎnghuì</t>
+  </si>
+  <si>
+    <t>Keep a low profile / conceal your talents and bide your time</t>
+  </si>
+  <si>
+    <t>Competitivness</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -233,6 +339,17 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="DengXian"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF5F6368"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -254,12 +371,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
@@ -540,7 +659,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:E12"/>
+  <dimension ref="B1:E13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="21.7109375" customWidth="1"/>
@@ -660,8 +779,166 @@
         <v>28</v>
       </c>
     </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" t="s">
+        <v>30</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12D0A2DA-AB68-4366-8798-7A63CA4E43F0}">
+  <dimension ref="B1:E10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="21" customWidth="1"/>
+    <col min="4" max="4" width="66" customWidth="1"/>
+    <col min="5" max="5" width="20.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B1" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B2" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B4" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B5" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" t="s">
+        <v>41</v>
+      </c>
+      <c r="E6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B7" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" t="s">
+        <v>51</v>
+      </c>
+      <c r="E7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B8" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B9" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" t="s">
+        <v>59</v>
+      </c>
+      <c r="E9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="D10" t="s">
+        <v>62</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chapter 2 of the Leadership and the rise of great powers
</commit_message>
<xml_diff>
--- a/Unusual words.xlsx
+++ b/Unusual words.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\InternationalRelations\International relations- notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C37206D9-929B-4011-8DF5-ED55F8252867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9216542-8351-4659-853D-16B14AD443DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2835" yWindow="3270" windowWidth="21600" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="68">
   <si>
     <t>juxtaposition</t>
   </si>
@@ -298,6 +298,18 @@
   </si>
   <si>
     <t>Competitivness</t>
+  </si>
+  <si>
+    <t>rectify</t>
+  </si>
+  <si>
+    <t>korygować</t>
+  </si>
+  <si>
+    <t>Corollaries</t>
+  </si>
+  <si>
+    <t>wnioski</t>
   </si>
 </sst>
 </file>
@@ -659,7 +671,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:E13"/>
+  <dimension ref="B1:E15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="21.7109375" customWidth="1"/>
@@ -788,6 +800,22 @@
       </c>
       <c r="E13" s="2" t="s">
         <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>66</v>
+      </c>
+      <c r="C15" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chapter 7 and 8
</commit_message>
<xml_diff>
--- a/Unusual words.xlsx
+++ b/Unusual words.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\InternationalRelations\International relations- notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2472F331-1B10-4BD5-B75E-C7D4143F850B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5C35E53-FDD7-4E39-8786-1E0CD6122C4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2835" yWindow="3270" windowWidth="21600" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="72">
   <si>
     <t>juxtaposition</t>
   </si>
@@ -316,6 +316,12 @@
   </si>
   <si>
     <t>istny/prawdziwy</t>
+  </si>
+  <si>
+    <t>Enfeoffment</t>
+  </si>
+  <si>
+    <t>system feudalny??</t>
   </si>
 </sst>
 </file>
@@ -677,7 +683,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:E16"/>
+  <dimension ref="B1:E17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="21.7109375" customWidth="1"/>
@@ -830,6 +836,14 @@
       </c>
       <c r="C16" t="s">
         <v>69</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>